<commit_message>
function to make ice plots. Works fine. Need to refine it now.
</commit_message>
<xml_diff>
--- a/FT_reaction_ML_project/complete_workflow_scripts/features.xlsx
+++ b/FT_reaction_ML_project/complete_workflow_scripts/features.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/hiregangea_cardiff_ac_uk/Documents/Desktop/personal_projects/FT_reaction_ML_project/catalyst_performance_optimizer/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/hiregangea_cardiff_ac_uk/Documents/Desktop/personal_projects/FT_reaction_ML_project/complete_workflow_scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="11_F25DC773A252ABDACC104873399A41685BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08A1C8E8-256F-451C-AED8-8FFBA20F1983}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="11_F25DC773A252ABDACC104873399A41685BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86AED2F9-9B7E-4AE2-9BE7-E5337695D8CF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,9 +31,6 @@
   </si>
   <si>
     <t>dCo, nm</t>
-  </si>
-  <si>
-    <t>BET, m^2/g</t>
   </si>
   <si>
     <t>Pt,Au,Ru %</t>
@@ -73,6 +70,9 @@
   </si>
   <si>
     <t>GHSV, L*h-1*g-1</t>
+  </si>
+  <si>
+    <t>BET, m^2 g-1</t>
   </si>
 </sst>
 </file>
@@ -195,10 +195,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -478,46 +474,46 @@
         <v>1</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="I1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>14</v>
       </c>
       <c r="S1" s="9"/>
       <c r="T1" s="9"/>

</xml_diff>